<commit_message>
chore: update daily market scan
</commit_message>
<xml_diff>
--- a/output/minervini_4h.xlsx
+++ b/output/minervini_4h.xlsx
@@ -1114,10 +1114,10 @@
         <v>817.5499877929688</v>
       </c>
       <c r="I9" t="n">
-        <v>262.023880250306</v>
+        <v>262.0239102537355</v>
       </c>
       <c r="J9" t="n">
-        <v>193.4083668475369</v>
+        <v>193.4083332503845</v>
       </c>
       <c r="K9" t="n">
         <v>6.341051089236993</v>
@@ -1268,10 +1268,10 @@
         <v>1982</v>
       </c>
       <c r="I11" t="n">
-        <v>821.6033372206257</v>
+        <v>821.6033975811163</v>
       </c>
       <c r="J11" t="n">
-        <v>137.8276610474978</v>
+        <v>137.8276435750843</v>
       </c>
       <c r="K11" t="n">
         <v>1.432958034800413</v>
@@ -13123,7 +13123,7 @@
         <v>3.164802535849276</v>
       </c>
       <c r="H165" t="n">
-        <v>2269.472002658311</v>
+        <v>2269.472253037084</v>
       </c>
       <c r="I165" t="n">
         <v>1353.205955540699</v>
@@ -13132,7 +13132,7 @@
         <v>57.77347056878131</v>
       </c>
       <c r="K165" t="n">
-        <v>6.298454457063762</v>
+        <v>6.298466184406726</v>
       </c>
       <c r="L165" t="n">
         <v>69.86111111111111</v>
@@ -15128,10 +15128,10 @@
         <v>2983.800048828125</v>
       </c>
       <c r="I191" t="n">
-        <v>1175.257470329055</v>
+        <v>1175.257587358084</v>
       </c>
       <c r="J191" t="n">
-        <v>108.5330330333436</v>
+        <v>108.533012268178</v>
       </c>
       <c r="K191" t="n">
         <v>21.74800021955521</v>
@@ -19283,7 +19283,7 @@
         <v>1.002257089081349</v>
       </c>
       <c r="H245" t="n">
-        <v>6552.654707500795</v>
+        <v>6552.654210942315</v>
       </c>
       <c r="I245" t="n">
         <v>4229.809203861739</v>
@@ -19292,7 +19292,7 @@
         <v>28.04360052588875</v>
       </c>
       <c r="K245" t="n">
-        <v>20.98697761264392</v>
+        <v>20.98696844428205</v>
       </c>
       <c r="L245" t="n">
         <v>50.41666666666666</v>
@@ -21824,7 +21824,7 @@
         <v>2.347184464716623</v>
       </c>
       <c r="H278" t="n">
-        <v>5038.987542214121</v>
+        <v>5038.987051168056</v>
       </c>
       <c r="I278" t="n">
         <v>3669.905008549105</v>
@@ -21833,7 +21833,7 @@
         <v>24.73074887051945</v>
       </c>
       <c r="K278" t="n">
-        <v>10.08165029413701</v>
+        <v>10.08163956675163</v>
       </c>
       <c r="L278" t="n">
         <v>51.38888888888889</v>
@@ -23136,10 +23136,10 @@
         <v>2295</v>
       </c>
       <c r="I295" t="n">
-        <v>1174.091384580817</v>
+        <v>1174.091262727543</v>
       </c>
       <c r="J295" t="n">
-        <v>67.11646140615035</v>
+        <v>67.11647875036249</v>
       </c>
       <c r="K295" t="n">
         <v>16.96651692351452</v>
@@ -23829,10 +23829,10 @@
         <v>529.9163379046904</v>
       </c>
       <c r="I304" t="n">
-        <v>387.2369934418427</v>
+        <v>387.2369630771774</v>
       </c>
       <c r="J304" t="n">
-        <v>22.84467141915105</v>
+        <v>22.84468105185065</v>
       </c>
       <c r="K304" t="n">
         <v>11.39716718654686</v>
@@ -28369,7 +28369,7 @@
         <v>-0.565653745454453</v>
       </c>
       <c r="H363" t="n">
-        <v>5875.534417311879</v>
+        <v>5875.533923201399</v>
       </c>
       <c r="I363" t="n">
         <v>5051</v>
@@ -28378,7 +28378,7 @@
         <v>8.226093842803394</v>
       </c>
       <c r="K363" t="n">
-        <v>7.482565029029153</v>
+        <v>7.482555990147244</v>
       </c>
       <c r="L363" t="n">
         <v>49.72222222222222</v>
@@ -30374,10 +30374,10 @@
         <v>443.3731066930094</v>
       </c>
       <c r="I389" t="n">
-        <v>191.8556220656042</v>
+        <v>191.8556371798532</v>
       </c>
       <c r="J389" t="n">
-        <v>82.68946003581175</v>
+        <v>82.68944564366755</v>
       </c>
       <c r="K389" t="n">
         <v>26.4973200265362</v>
@@ -32835,7 +32835,7 @@
         <v>-0.3878305876905075</v>
       </c>
       <c r="H421" t="n">
-        <v>45150.85152546577</v>
+        <v>45150.8475731383</v>
       </c>
       <c r="I421" t="n">
         <v>29525.27356749276</v>
@@ -32844,7 +32844,7 @@
         <v>23.28420909222768</v>
       </c>
       <c r="K421" t="n">
-        <v>24.04080089413674</v>
+        <v>24.04079003609423</v>
       </c>
       <c r="L421" t="n">
         <v>36.52777777777778</v>
@@ -36223,7 +36223,7 @@
         <v>0.7567775940050536</v>
       </c>
       <c r="H465" t="n">
-        <v>848.8262434052705</v>
+        <v>848.8263047717415</v>
       </c>
       <c r="I465" t="n">
         <v>495.5999980879241</v>
@@ -36232,7 +36232,7 @@
         <v>21.87247827487777</v>
       </c>
       <c r="K465" t="n">
-        <v>40.53414625915075</v>
+        <v>40.53415641916251</v>
       </c>
       <c r="L465" t="n">
         <v>37.63888888888889</v>
@@ -36842,10 +36842,10 @@
         <v>286.0804516993438</v>
       </c>
       <c r="I473" t="n">
-        <v>171.9528178807998</v>
+        <v>171.952833032562</v>
       </c>
       <c r="J473" t="n">
-        <v>22.06836531285579</v>
+        <v>22.06835455670364</v>
       </c>
       <c r="K473" t="n">
         <v>36.29369224299695</v>
@@ -37455,7 +37455,7 @@
         <v>1.157518369471844</v>
       </c>
       <c r="H481" t="n">
-        <v>329.6445669998864</v>
+        <v>329.6445362713373</v>
       </c>
       <c r="I481" t="n">
         <v>191.2413512696417</v>
@@ -37464,7 +37464,7 @@
         <v>24.28274068230316</v>
       </c>
       <c r="K481" t="n">
-        <v>38.69260230479468</v>
+        <v>38.69258937625628</v>
       </c>
       <c r="L481" t="n">
         <v>25.97222222222222</v>
@@ -38841,7 +38841,7 @@
         <v>-1.134908059779705</v>
       </c>
       <c r="H499" t="n">
-        <v>478.7148398145708</v>
+        <v>478.7148709533388</v>
       </c>
       <c r="I499" t="n">
         <v>355.1755291130353</v>
@@ -38850,7 +38850,7 @@
         <v>15.40772387109837</v>
       </c>
       <c r="K499" t="n">
-        <v>16.78820369425642</v>
+        <v>16.78821129093084</v>
       </c>
       <c r="L499" t="n">
         <v>54.72222222222223</v>
@@ -40153,10 +40153,10 @@
         <v>555.1842484654879</v>
       </c>
       <c r="I516" t="n">
-        <v>379.7398698331913</v>
+        <v>379.7399002549519</v>
       </c>
       <c r="J516" t="n">
-        <v>11.11554138162569</v>
+        <v>11.1155324799264</v>
       </c>
       <c r="K516" t="n">
         <v>31.57583419930909</v>
@@ -40997,7 +40997,7 @@
         <v>-0.6210973687980514</v>
       </c>
       <c r="H527" t="n">
-        <v>163308.4863287346</v>
+        <v>163308.5022863474</v>
       </c>
       <c r="I527" t="n">
         <v>121787.4350540836</v>
@@ -41006,7 +41006,7 @@
         <v>3.187984823058465</v>
       </c>
       <c r="K527" t="n">
-        <v>29.95025569247602</v>
+        <v>29.95026839050485</v>
       </c>
       <c r="L527" t="n">
         <v>27.91666666666667</v>
@@ -44542,10 +44542,10 @@
         <v>409.9712889887167</v>
       </c>
       <c r="I573" t="n">
-        <v>309.8384816659088</v>
+        <v>309.838511773213</v>
       </c>
       <c r="J573" t="n">
-        <v>4.457649081003479</v>
+        <v>4.457638930753949</v>
       </c>
       <c r="K573" t="n">
         <v>26.67118699833535</v>
@@ -46233,16 +46233,16 @@
         <v>-1.045338384895489</v>
       </c>
       <c r="H595" t="n">
-        <v>239.2187037807859</v>
+        <v>239.2186883393384</v>
       </c>
       <c r="I595" t="n">
-        <v>156.7443123050878</v>
+        <v>156.7442971017576</v>
       </c>
       <c r="J595" t="n">
-        <v>12.28477602264306</v>
+        <v>12.28478691364554</v>
       </c>
       <c r="K595" t="n">
-        <v>35.91971805726472</v>
+        <v>35.91970928371502</v>
       </c>
       <c r="L595" t="n">
         <v>26.52777777777778</v>
@@ -46849,7 +46849,7 @@
         <v>-1.355180243355558</v>
       </c>
       <c r="H603" t="n">
-        <v>155.8999606999571</v>
+        <v>155.8999783750524</v>
       </c>
       <c r="I603" t="n">
         <v>110.3499984741211</v>
@@ -46858,7 +46858,7 @@
         <v>4.630721052116682</v>
       </c>
       <c r="K603" t="n">
-        <v>35.02508395647732</v>
+        <v>35.02509926489184</v>
       </c>
       <c r="L603" t="n">
         <v>24.16666666666667</v>
@@ -48851,7 +48851,7 @@
         <v>-0.5289877462034021</v>
       </c>
       <c r="H629" t="n">
-        <v>632.5129117162858</v>
+        <v>632.5128493651639</v>
       </c>
       <c r="I629" t="n">
         <v>351.0001816860465</v>
@@ -48860,7 +48860,7 @@
         <v>19.99994136292933</v>
       </c>
       <c r="K629" t="n">
-        <v>50.16925294042692</v>
+        <v>50.16923813721701</v>
       </c>
       <c r="L629" t="n">
         <v>17.08333333333333</v>
@@ -49621,7 +49621,7 @@
         <v>-1.434342585985138</v>
       </c>
       <c r="H639" t="n">
-        <v>1608.140814494163</v>
+        <v>1608.140938678776</v>
       </c>
       <c r="I639" t="n">
         <v>1081.099975585938</v>
@@ -49630,7 +49630,7 @@
         <v>4.745171583259111</v>
       </c>
       <c r="K639" t="n">
-        <v>42.01172552307764</v>
+        <v>42.0117364895745</v>
       </c>
       <c r="L639" t="n">
         <v>15.69444444444444</v>
@@ -49698,7 +49698,7 @@
         <v>-1.666775813593147</v>
       </c>
       <c r="H640" t="n">
-        <v>154.1041584954392</v>
+        <v>154.1041427094461</v>
       </c>
       <c r="I640" t="n">
         <v>104.7068431385872</v>
@@ -49707,7 +49707,7 @@
         <v>4.176573909958581</v>
       </c>
       <c r="K640" t="n">
-        <v>41.27627054326495</v>
+        <v>41.27625607132437</v>
       </c>
       <c r="L640" t="n">
         <v>15.55555555555556</v>
@@ -49852,7 +49852,7 @@
         <v>-0.824073811416659</v>
       </c>
       <c r="H642" t="n">
-        <v>308.0746526166167</v>
+        <v>308.0746845932235</v>
       </c>
       <c r="I642" t="n">
         <v>185.2067002350832</v>
@@ -49861,7 +49861,7 @@
         <v>13.72158504516692</v>
       </c>
       <c r="K642" t="n">
-        <v>46.2703730693784</v>
+        <v>46.27038825151091</v>
       </c>
       <c r="L642" t="n">
         <v>15.27777777777778</v>
@@ -50160,7 +50160,7 @@
         <v>-0.911543638119694</v>
       </c>
       <c r="H646" t="n">
-        <v>124.8273017901132</v>
+        <v>124.8273096544699</v>
       </c>
       <c r="I646" t="n">
         <v>76.65010804466255</v>
@@ -50169,7 +50169,7 @@
         <v>7.501481247575037</v>
       </c>
       <c r="K646" t="n">
-        <v>51.48944111476668</v>
+        <v>51.48945065888879</v>
       </c>
       <c r="L646" t="n">
         <v>14.58333333333333</v>
@@ -50314,7 +50314,7 @@
         <v>-1.956888492501585</v>
       </c>
       <c r="H648" t="n">
-        <v>398.263766662724</v>
+        <v>398.2637357690495</v>
       </c>
       <c r="I648" t="n">
         <v>243.9284560598348</v>
@@ -50323,7 +50323,7 @@
         <v>9.048367827471161</v>
       </c>
       <c r="K648" t="n">
-        <v>49.72322054989626</v>
+        <v>49.7232089357329</v>
       </c>
       <c r="L648" t="n">
         <v>14.30555555555556</v>
@@ -51084,7 +51084,7 @@
         <v>-3.066272652257995</v>
       </c>
       <c r="H658" t="n">
-        <v>1255.178432949836</v>
+        <v>1255.178308316206</v>
       </c>
       <c r="I658" t="n">
         <v>855.1500244140625</v>
@@ -51093,7 +51093,7 @@
         <v>2.905919999588891</v>
       </c>
       <c r="K658" t="n">
-        <v>42.63391283520865</v>
+        <v>42.63389867229614</v>
       </c>
       <c r="L658" t="n">
         <v>11.80555555555556</v>
@@ -51546,7 +51546,7 @@
         <v>-2.188923610668525</v>
       </c>
       <c r="H664" t="n">
-        <v>729.6617501297184</v>
+        <v>729.6618113637422</v>
       </c>
       <c r="I664" t="n">
         <v>446.5</v>
@@ -51555,7 +51555,7 @@
         <v>6.830907054871216</v>
       </c>
       <c r="K664" t="n">
-        <v>52.9689203626244</v>
+        <v>52.96893319994596</v>
       </c>
       <c r="L664" t="n">
         <v>10.69444444444444</v>
@@ -51700,7 +51700,7 @@
         <v>-2.604193874278637</v>
       </c>
       <c r="H666" t="n">
-        <v>263.2205288662585</v>
+        <v>263.220498300555</v>
       </c>
       <c r="I666" t="n">
         <v>163.3000030517578</v>
@@ -51709,7 +51709,7 @@
         <v>2.161664858131118</v>
       </c>
       <c r="K666" t="n">
-        <v>57.77769344677972</v>
+        <v>57.77767512531289</v>
       </c>
       <c r="L666" t="n">
         <v>10.13888888888889</v>
@@ -51777,7 +51777,7 @@
         <v>-2.148565704371641</v>
       </c>
       <c r="H667" t="n">
-        <v>406.5707642578344</v>
+        <v>406.5707952146441</v>
       </c>
       <c r="I667" t="n">
         <v>255.5</v>
@@ -51786,7 +51786,7 @@
         <v>2.661443363197158</v>
       </c>
       <c r="K667" t="n">
-        <v>55.00220479565458</v>
+        <v>55.00221659771753</v>
       </c>
       <c r="L667" t="n">
         <v>10</v>
@@ -52316,7 +52316,7 @@
         <v>-1.394065988772819</v>
       </c>
       <c r="H674" t="n">
-        <v>1211.101032727737</v>
+        <v>1211.101157071308</v>
       </c>
       <c r="I674" t="n">
         <v>577.3964738257137</v>
@@ -52325,7 +52325,7 @@
         <v>12.05471964750795</v>
       </c>
       <c r="K674" t="n">
-        <v>87.18717661943391</v>
+        <v>87.18719583791471</v>
       </c>
       <c r="L674" t="n">
         <v>8.611111111111111</v>
@@ -54010,7 +54010,7 @@
         <v>-1.677722712351626</v>
       </c>
       <c r="H696" t="n">
-        <v>891.9600709299998</v>
+        <v>891.9600088223455</v>
       </c>
       <c r="I696" t="n">
         <v>455</v>
@@ -54019,7 +54019,7 @@
         <v>1.516482175051515</v>
       </c>
       <c r="K696" t="n">
-        <v>93.10675096694101</v>
+        <v>93.1067375208152</v>
       </c>
       <c r="L696" t="n">
         <v>3.611111111111111</v>

</xml_diff>